<commit_message>
Update test reference files: when sorting rows and sort columns produce 'duplicate rows', leave order unchanged from original. Example sorting by columns 1 and 2 should leave this unchanged: A a b A a A
</commit_message>
<xml_diff>
--- a/ClosedXML.Tests/Resource/Examples/AutoFilter/RegularAutoFilter.xlsx
+++ b/ClosedXML.Tests/Resource/Examples/AutoFilter/RegularAutoFilter.xlsx
@@ -31,10 +31,10 @@
     <x:t>Names</x:t>
   </x:si>
   <x:si>
+    <x:t>Alex</x:t>
+  </x:si>
+  <x:si>
     <x:t>Jacques</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Alex</x:t>
   </x:si>
   <x:si>
     <x:t>Patrick</x:t>
@@ -453,7 +453,7 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" spans="1:2">
+    <x:row r="2" spans="1:2" hidden="1">
       <x:c r="A2" s="0" t="n">
         <x:v>5</x:v>
       </x:c>
@@ -461,7 +461,7 @@
         <x:v>2</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" spans="1:2" hidden="1">
+    <x:row r="3" spans="1:2">
       <x:c r="A3" s="0" t="n">
         <x:v>5</x:v>
       </x:c>

</xml_diff>